<commit_message>
update docker image and orther
</commit_message>
<xml_diff>
--- a/write-file/receipt.xlsx
+++ b/write-file/receipt.xlsx
@@ -440,12 +440,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -456,7 +456,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>บริษัท บิ๊กซี ซูเปอร์เซ็นเตอร์ จำกัด (มหาชน)</t>
+          <t>บริษัท เอก-ชัย ดีสทริบิวชั่น ซิสเทม จำกัด</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr"/>
@@ -517,29 +517,25 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>8850718810529</t>
+          <t>08851932354110</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>เลย์ร็อคกุ้งเผาซีฟุ๊ด69ก (หน่วย:1ชิ้น)</t>
+          <t>ร ซันซิลแชมพู แดเมจรีสโตร์ an 60มล</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr"/>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>31.00</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+          <t>20.000</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr"/>
       <c r="G3" s="1" t="inlineStr"/>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>31.00</t>
+          <t>20.00 บ</t>
         </is>
       </c>
     </row>
@@ -551,29 +547,25 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>6923655599009</t>
+          <t>06920890700610</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>ดินสอกด 0.5 G990 PK1 (หน่วย:1ชิ้น)</t>
+          <t>จูปาจุปส์ออริจินอล 9.5n.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr"/>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>14.00</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+          <t>5.000</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr"/>
       <c r="G4" s="1" t="inlineStr"/>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>14.00</t>
+          <t>5.00 บ</t>
         </is>
       </c>
     </row>
@@ -585,47 +577,133 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>8852023664675</t>
+          <t>08850999321004</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>โก๋แก่หิมพานต์อบเกลือ 30ก.(หน่วย:1ชิ้น)</t>
+          <t>8 สิงห์น้าดื่ม 600มล.</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr"/>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>25.00</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
+          <t>7.000</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr"/>
       <c r="G5" s="1" t="inlineStr"/>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>25.00</t>
+          <t>7.00 บ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>ยอดเงินชำระ</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr"/>
-      <c r="C6" s="1" t="inlineStr"/>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>08935001723073</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>จูปาจุปส์ดิปแอนด์ลิค 9 n.</t>
+        </is>
+      </c>
       <c r="D6" s="1" t="inlineStr"/>
-      <c r="E6" s="1" t="inlineStr"/>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>7.000</t>
+        </is>
+      </c>
       <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>70.00</t>
+          <t>7.00 บ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>03046920029582</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Aun เอ็กเซอร์แลนซ์ดาร์ก 85% โกโก้35ก.</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr"/>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>49.000</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr"/>
+      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>49.00 บ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>09556001027252</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>คิทแคทชอคโกแลตพรีเมียม 35n.</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr"/>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>28.000</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr"/>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>28.00 บ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>ยอดเงินชำระ</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr"/>
+      <c r="C9" s="1" t="inlineStr"/>
+      <c r="D9" s="1" t="inlineStr"/>
+      <c r="E9" s="1" t="inlineStr"/>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>116.00</t>
         </is>
       </c>
     </row>

</xml_diff>